<commit_message>
Auto update Pengadaan 2026-10-26 08:48:44
</commit_message>
<xml_diff>
--- a/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-26).xlsx
+++ b/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-26).xlsx
@@ -1294,13 +1294,13 @@
         <v>17</v>
       </c>
       <c r="D24" s="10" t="n">
-        <v>338217900</v>
+        <v>350423349</v>
       </c>
       <c r="E24" s="8" t="n">
         <v>17</v>
       </c>
       <c r="F24" s="10" t="n">
-        <v>338217900</v>
+        <v>350423349</v>
       </c>
       <c r="G24" s="8" t="n">
         <v>17</v>
@@ -1332,13 +1332,13 @@
         <v>41</v>
       </c>
       <c r="D25" s="6" t="n">
-        <v>338324988</v>
+        <v>351115088</v>
       </c>
       <c r="E25" s="4" t="n">
         <v>40</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>293896298</v>
+        <v>306686398</v>
       </c>
       <c r="G25" s="4" t="n">
         <v>40</v>
@@ -1776,13 +1776,13 @@
         <v>27</v>
       </c>
       <c r="D37" s="6" t="n">
-        <v>391109425</v>
+        <v>418306096</v>
       </c>
       <c r="E37" s="4" t="n">
         <v>27</v>
       </c>
       <c r="F37" s="6" t="n">
-        <v>391109425</v>
+        <v>418306096</v>
       </c>
       <c r="G37" s="4" t="n">
         <v>27</v>
@@ -1852,13 +1852,13 @@
         <v>20</v>
       </c>
       <c r="D39" s="6" t="n">
-        <v>78370717</v>
+        <v>132336493</v>
       </c>
       <c r="E39" s="4" t="n">
         <v>20</v>
       </c>
       <c r="F39" s="6" t="n">
-        <v>78370717</v>
+        <v>132336493</v>
       </c>
       <c r="G39" s="4" t="n">
         <v>20</v>
@@ -2051,10 +2051,10 @@
         </is>
       </c>
       <c r="C44" s="8" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D44" s="10" t="n">
-        <v>159724173</v>
+        <v>147600173</v>
       </c>
       <c r="E44" s="11" t="inlineStr">
         <is>
@@ -2077,10 +2077,10 @@
         </is>
       </c>
       <c r="I44" s="8" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="J44" s="10" t="n">
-        <v>159724173</v>
+        <v>147600173</v>
       </c>
     </row>
     <row r="45" ht="45" customHeight="1">
@@ -2093,10 +2093,10 @@
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="D45" s="6" t="n">
-        <v>627367735</v>
+        <v>614397985</v>
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
@@ -2119,10 +2119,10 @@
         </is>
       </c>
       <c r="I45" s="4" t="n">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="J45" s="6" t="n">
-        <v>627367735</v>
+        <v>614397985</v>
       </c>
     </row>
     <row r="46" ht="45" customHeight="1">
@@ -2597,10 +2597,10 @@
         </is>
       </c>
       <c r="C57" s="4" t="n">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D57" s="6" t="n">
-        <v>871402790</v>
+        <v>848169190</v>
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
@@ -2623,10 +2623,10 @@
         </is>
       </c>
       <c r="I57" s="4" t="n">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="J57" s="6" t="n">
-        <v>871402790</v>
+        <v>848169190</v>
       </c>
     </row>
     <row r="58" ht="45" customHeight="1">
@@ -2681,10 +2681,10 @@
         </is>
       </c>
       <c r="C59" s="4" t="n">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D59" s="6" t="n">
-        <v>829576296</v>
+        <v>825988296</v>
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
@@ -2707,10 +2707,10 @@
         </is>
       </c>
       <c r="I59" s="4" t="n">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="J59" s="6" t="n">
-        <v>829576296</v>
+        <v>825988296</v>
       </c>
     </row>
     <row r="60" ht="45" customHeight="1">
@@ -3444,13 +3444,13 @@
         <v>13</v>
       </c>
       <c r="D77" s="6" t="n">
-        <v>35845048</v>
+        <v>66380633</v>
       </c>
       <c r="E77" s="4" t="n">
         <v>13</v>
       </c>
       <c r="F77" s="6" t="n">
-        <v>35845048</v>
+        <v>66380633</v>
       </c>
       <c r="G77" s="4" t="n">
         <v>13</v>
@@ -3983,10 +3983,10 @@
         </is>
       </c>
       <c r="C90" s="8" t="n">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="D90" s="10" t="n">
-        <v>164225425</v>
+        <v>130909625</v>
       </c>
       <c r="E90" s="11" t="inlineStr">
         <is>
@@ -4009,10 +4009,10 @@
         </is>
       </c>
       <c r="I90" s="8" t="n">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="J90" s="10" t="n">
-        <v>164225425</v>
+        <v>130909625</v>
       </c>
     </row>
     <row r="91" ht="45" customHeight="1">
@@ -4432,13 +4432,13 @@
         <v>31</v>
       </c>
       <c r="D101" s="6" t="n">
-        <v>207985114</v>
+        <v>238180114</v>
       </c>
       <c r="E101" s="4" t="n">
         <v>31</v>
       </c>
       <c r="F101" s="6" t="n">
-        <v>207985114</v>
+        <v>238180114</v>
       </c>
       <c r="G101" s="4" t="n">
         <v>31</v>
@@ -4589,10 +4589,10 @@
         </is>
       </c>
       <c r="C105" s="4" t="n">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="D105" s="6" t="n">
-        <v>1284304356</v>
+        <v>1258579356</v>
       </c>
       <c r="E105" s="7" t="inlineStr">
         <is>
@@ -4615,10 +4615,10 @@
         </is>
       </c>
       <c r="I105" s="4" t="n">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="J105" s="6" t="n">
-        <v>1284304356</v>
+        <v>1258579356</v>
       </c>
     </row>
     <row r="106" ht="45" customHeight="1">
@@ -4629,16 +4629,16 @@
         </is>
       </c>
       <c r="C106" s="12" t="n">
-        <v>4023</v>
+        <v>3996</v>
       </c>
       <c r="D106" s="13" t="n">
-        <v>34505997953</v>
+        <v>34561930384</v>
       </c>
       <c r="E106" s="12" t="n">
         <v>564</v>
       </c>
       <c r="F106" s="13" t="n">
-        <v>7770758287</v>
+        <v>7937646868</v>
       </c>
       <c r="G106" s="12" t="n">
         <v>564</v>
@@ -4647,10 +4647,10 @@
         <v>7047187293</v>
       </c>
       <c r="I106" s="12" t="n">
-        <v>3459</v>
+        <v>3432</v>
       </c>
       <c r="J106" s="13" t="n">
-        <v>26735239666</v>
+        <v>26624283516</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update Pengadaan 2026-10-26 13:14:18
</commit_message>
<xml_diff>
--- a/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-26).xlsx
+++ b/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-26).xlsx
@@ -894,13 +894,13 @@
         <v>2</v>
       </c>
       <c r="D14" s="10" t="n">
-        <v>63250745</v>
+        <v>63250744</v>
       </c>
       <c r="E14" s="8" t="n">
         <v>2</v>
       </c>
       <c r="F14" s="10" t="n">
-        <v>63250745</v>
+        <v>63250744</v>
       </c>
       <c r="G14" s="8" t="n">
         <v>2</v>
@@ -1184,13 +1184,13 @@
         <v>7</v>
       </c>
       <c r="D21" s="6" t="n">
-        <v>61019294</v>
+        <v>63785294</v>
       </c>
       <c r="E21" s="4" t="n">
         <v>6</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>55769294</v>
+        <v>58535294</v>
       </c>
       <c r="G21" s="4" t="n">
         <v>6</v>
@@ -1215,22 +1215,22 @@
         </is>
       </c>
       <c r="C22" s="8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D22" s="10" t="n">
-        <v>84907554</v>
+        <v>74152766</v>
       </c>
       <c r="E22" s="8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F22" s="10" t="n">
-        <v>84907554</v>
+        <v>74152766</v>
       </c>
       <c r="G22" s="8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H22" s="10" t="n">
-        <v>78869208</v>
+        <v>128214258</v>
       </c>
       <c r="I22" s="11" t="inlineStr">
         <is>
@@ -1253,22 +1253,22 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="D23" s="6" t="n">
-        <v>137583844</v>
+        <v>136080290</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>137583844</v>
+        <v>136080290</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>13</v>
+        <v>40</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>116218702</v>
+        <v>1520271914</v>
       </c>
       <c r="I23" s="7" t="inlineStr">
         <is>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="C24" s="8" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D24" s="10" t="n">
-        <v>350423349</v>
+        <v>340118400</v>
       </c>
       <c r="E24" s="8" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F24" s="10" t="n">
-        <v>350423349</v>
+        <v>340118400</v>
       </c>
       <c r="G24" s="8" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H24" s="10" t="n">
-        <v>350174900</v>
+        <v>3049472900</v>
       </c>
       <c r="I24" s="11" t="inlineStr">
         <is>
@@ -1329,22 +1329,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
+        <v>42</v>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>351294738</v>
+      </c>
+      <c r="E25" s="4" t="n">
         <v>41</v>
       </c>
-      <c r="D25" s="6" t="n">
-        <v>351115088</v>
-      </c>
-      <c r="E25" s="4" t="n">
-        <v>40</v>
-      </c>
       <c r="F25" s="6" t="n">
-        <v>306686398</v>
+        <v>306866048</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>282976443</v>
+        <v>398476383</v>
       </c>
       <c r="I25" s="4" t="n">
         <v>1</v>
@@ -1366,13 +1366,13 @@
         <v>1</v>
       </c>
       <c r="D26" s="10" t="n">
-        <v>38508000</v>
+        <v>28881000</v>
       </c>
       <c r="E26" s="8" t="n">
         <v>1</v>
       </c>
       <c r="F26" s="10" t="n">
-        <v>38508000</v>
+        <v>28881000</v>
       </c>
       <c r="G26" s="8" t="n">
         <v>1</v>
@@ -1401,22 +1401,22 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D27" s="6" t="n">
-        <v>1228508400</v>
+        <v>1219004247</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F27" s="6" t="n">
-        <v>1228508400</v>
+        <v>1219004247</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>1207367631</v>
+        <v>3076832926</v>
       </c>
       <c r="I27" s="7" t="inlineStr">
         <is>
@@ -1439,22 +1439,22 @@
         </is>
       </c>
       <c r="C28" s="8" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D28" s="10" t="n">
         <v>90550292</v>
       </c>
       <c r="E28" s="8" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F28" s="10" t="n">
         <v>90550292</v>
       </c>
       <c r="G28" s="8" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H28" s="10" t="n">
-        <v>86612607</v>
+        <v>236612607</v>
       </c>
       <c r="I28" s="11" t="inlineStr">
         <is>
@@ -1480,25 +1480,29 @@
         <v>14</v>
       </c>
       <c r="D29" s="6" t="n">
-        <v>65316100</v>
+        <v>65172075</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F29" s="6" t="n">
-        <v>50379150</v>
+        <v>65172075</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="H29" s="6" t="n">
-        <v>46526860</v>
-      </c>
-      <c r="I29" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="J29" s="6" t="n">
-        <v>14936950</v>
+        <v>61364960</v>
+      </c>
+      <c r="I29" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J29" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="30" ht="45" customHeight="1">
@@ -1514,13 +1518,13 @@
         <v>6</v>
       </c>
       <c r="D30" s="10" t="n">
-        <v>107342366</v>
+        <v>103722907</v>
       </c>
       <c r="E30" s="8" t="n">
         <v>6</v>
       </c>
       <c r="F30" s="10" t="n">
-        <v>107342366</v>
+        <v>103722907</v>
       </c>
       <c r="G30" s="8" t="n">
         <v>6</v>
@@ -1552,13 +1556,13 @@
         <v>5</v>
       </c>
       <c r="D31" s="6" t="n">
-        <v>108974684</v>
+        <v>20641550</v>
       </c>
       <c r="E31" s="4" t="n">
         <v>5</v>
       </c>
       <c r="F31" s="6" t="n">
-        <v>108974684</v>
+        <v>20641550</v>
       </c>
       <c r="G31" s="4" t="n">
         <v>5</v>
@@ -1628,13 +1632,13 @@
         <v>6</v>
       </c>
       <c r="D33" s="6" t="n">
-        <v>93366423</v>
+        <v>93231105</v>
       </c>
       <c r="E33" s="4" t="n">
         <v>6</v>
       </c>
       <c r="F33" s="6" t="n">
-        <v>93366423</v>
+        <v>93231105</v>
       </c>
       <c r="G33" s="4" t="n">
         <v>6</v>
@@ -1666,13 +1670,13 @@
         <v>13</v>
       </c>
       <c r="D34" s="10" t="n">
-        <v>334343818</v>
+        <v>333822118</v>
       </c>
       <c r="E34" s="8" t="n">
         <v>13</v>
       </c>
       <c r="F34" s="10" t="n">
-        <v>334343818</v>
+        <v>333822118</v>
       </c>
       <c r="G34" s="8" t="n">
         <v>13</v>
@@ -1701,28 +1705,30 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="D35" s="6" t="n">
-        <v>461686502</v>
+        <v>224284602</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="F35" s="6" t="n">
-        <v>412496502</v>
+        <v>224284602</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="H35" s="6" t="n">
-        <v>402113040</v>
+        <v>5025718580</v>
       </c>
       <c r="I35" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="J35" s="6" t="n">
-        <v>49190000</v>
+        <v>4</v>
+      </c>
+      <c r="J35" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="36" ht="45" customHeight="1">
@@ -1738,13 +1744,13 @@
         <v>12</v>
       </c>
       <c r="D36" s="10" t="n">
-        <v>101993338</v>
+        <v>100392718</v>
       </c>
       <c r="E36" s="8" t="n">
         <v>12</v>
       </c>
       <c r="F36" s="10" t="n">
-        <v>101993338</v>
+        <v>100392718</v>
       </c>
       <c r="G36" s="8" t="n">
         <v>12</v>
@@ -1773,22 +1779,22 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D37" s="6" t="n">
-        <v>418306096</v>
+        <v>388813025</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F37" s="6" t="n">
-        <v>418306096</v>
+        <v>388813025</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H37" s="6" t="n">
-        <v>409964886</v>
+        <v>450041436</v>
       </c>
       <c r="I37" s="7" t="inlineStr">
         <is>
@@ -1852,13 +1858,13 @@
         <v>20</v>
       </c>
       <c r="D39" s="6" t="n">
-        <v>132336493</v>
+        <v>118968429</v>
       </c>
       <c r="E39" s="4" t="n">
         <v>20</v>
       </c>
       <c r="F39" s="6" t="n">
-        <v>132336493</v>
+        <v>118968429</v>
       </c>
       <c r="G39" s="4" t="n">
         <v>20</v>
@@ -2768,13 +2774,13 @@
         <v>3</v>
       </c>
       <c r="D61" s="6" t="n">
-        <v>34949904</v>
+        <v>54570486</v>
       </c>
       <c r="E61" s="4" t="n">
         <v>3</v>
       </c>
       <c r="F61" s="6" t="n">
-        <v>34949904</v>
+        <v>54570486</v>
       </c>
       <c r="G61" s="4" t="n">
         <v>3</v>
@@ -2803,22 +2809,22 @@
         </is>
       </c>
       <c r="C62" s="8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D62" s="10" t="n">
-        <v>151137140</v>
+        <v>80621140</v>
       </c>
       <c r="E62" s="8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F62" s="10" t="n">
-        <v>151137140</v>
+        <v>80621140</v>
       </c>
       <c r="G62" s="8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H62" s="10" t="n">
-        <v>72726534</v>
+        <v>83626512</v>
       </c>
       <c r="I62" s="11" t="inlineStr">
         <is>
@@ -2925,22 +2931,22 @@
         </is>
       </c>
       <c r="C65" s="4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D65" s="6" t="n">
-        <v>124972901</v>
+        <v>173625311</v>
       </c>
       <c r="E65" s="4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F65" s="6" t="n">
-        <v>124972901</v>
+        <v>173625311</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H65" s="6" t="n">
-        <v>121983128</v>
+        <v>318350703</v>
       </c>
       <c r="I65" s="7" t="inlineStr">
         <is>
@@ -2966,25 +2972,29 @@
         <v>31</v>
       </c>
       <c r="D66" s="10" t="n">
-        <v>278141173</v>
+        <v>276216173</v>
       </c>
       <c r="E66" s="8" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F66" s="10" t="n">
-        <v>274236748</v>
+        <v>276216173</v>
       </c>
       <c r="G66" s="8" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="H66" s="10" t="n">
-        <v>250171300</v>
-      </c>
-      <c r="I66" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="J66" s="10" t="n">
-        <v>3904425</v>
+        <v>253688800</v>
+      </c>
+      <c r="I66" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J66" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="67" ht="45" customHeight="1">
@@ -3298,35 +3308,27 @@
           <t>LABORATORIUM KESEHATAN DAERAH - 1.02.0.00.0.00.01.0003</t>
         </is>
       </c>
-      <c r="C74" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="C74" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="D74" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E74" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="E74" s="8" t="n">
+        <v>2</v>
       </c>
       <c r="F74" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G74" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H74" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G74" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H74" s="10" t="n">
+        <v>65401200</v>
       </c>
       <c r="I74" s="11" t="inlineStr">
         <is>
@@ -3444,13 +3446,13 @@
         <v>13</v>
       </c>
       <c r="D77" s="6" t="n">
-        <v>66380633</v>
+        <v>56639836</v>
       </c>
       <c r="E77" s="4" t="n">
         <v>13</v>
       </c>
       <c r="F77" s="6" t="n">
-        <v>66380633</v>
+        <v>56639836</v>
       </c>
       <c r="G77" s="4" t="n">
         <v>13</v>
@@ -4238,13 +4240,13 @@
         <v>2</v>
       </c>
       <c r="D96" s="10" t="n">
-        <v>35716900</v>
+        <v>28826575</v>
       </c>
       <c r="E96" s="8" t="n">
         <v>2</v>
       </c>
       <c r="F96" s="10" t="n">
-        <v>35716900</v>
+        <v>28826575</v>
       </c>
       <c r="G96" s="8" t="n">
         <v>2</v>
@@ -4273,22 +4275,22 @@
         </is>
       </c>
       <c r="C97" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D97" s="6" t="n">
         <v>108000000</v>
       </c>
       <c r="E97" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F97" s="6" t="n">
         <v>108000000</v>
       </c>
       <c r="G97" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H97" s="6" t="n">
-        <v>158730000</v>
+        <v>2359971000</v>
       </c>
       <c r="I97" s="7" t="inlineStr">
         <is>
@@ -4432,13 +4434,13 @@
         <v>31</v>
       </c>
       <c r="D101" s="6" t="n">
-        <v>238180114</v>
+        <v>222926114</v>
       </c>
       <c r="E101" s="4" t="n">
         <v>31</v>
       </c>
       <c r="F101" s="6" t="n">
-        <v>238180114</v>
+        <v>222926114</v>
       </c>
       <c r="G101" s="4" t="n">
         <v>31</v>
@@ -4629,28 +4631,28 @@
         </is>
       </c>
       <c r="C106" s="12" t="n">
-        <v>3996</v>
+        <v>4048</v>
       </c>
       <c r="D106" s="13" t="n">
-        <v>34561930384</v>
+        <v>34112511168</v>
       </c>
       <c r="E106" s="12" t="n">
-        <v>564</v>
+        <v>621</v>
       </c>
       <c r="F106" s="13" t="n">
-        <v>7937646868</v>
+        <v>7556259027</v>
       </c>
       <c r="G106" s="12" t="n">
-        <v>564</v>
+        <v>621</v>
       </c>
       <c r="H106" s="13" t="n">
-        <v>7047187293</v>
+        <v>20490796233</v>
       </c>
       <c r="I106" s="12" t="n">
-        <v>3432</v>
+        <v>3427</v>
       </c>
       <c r="J106" s="13" t="n">
-        <v>26624283516</v>
+        <v>26556252141</v>
       </c>
     </row>
   </sheetData>
@@ -5025,13 +5027,13 @@
         <v>3</v>
       </c>
       <c r="D10" s="10" t="n">
-        <v>276710330</v>
+        <v>261110330</v>
       </c>
       <c r="E10" s="8" t="n">
         <v>3</v>
       </c>
       <c r="F10" s="10" t="n">
-        <v>276710330</v>
+        <v>261110330</v>
       </c>
       <c r="G10" s="8" t="n">
         <v>3</v>
@@ -5709,35 +5711,55 @@
           <t>DINAS KEPENDUDUKAN DAN PENCATATAN SIPIL - 2.12.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C22" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D22" s="10" t="n">
-        <v>54773006</v>
-      </c>
-      <c r="E22" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F22" s="10" t="n">
-        <v>54773006</v>
-      </c>
-      <c r="G22" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="H22" s="10" t="n">
-        <v>49345050</v>
-      </c>
-      <c r="I22" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="J22" s="10" t="n">
-        <v>49345050</v>
-      </c>
-      <c r="K22" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="L22" s="10" t="n">
-        <v>49345050</v>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E22" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F22" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G22" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H22" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I22" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J22" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K22" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L22" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M22" s="11" t="inlineStr">
         <is>
@@ -5760,34 +5782,34 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D23" s="6" t="n">
-        <v>1225542538</v>
+        <v>1055829695</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>1225542538</v>
+        <v>1055829695</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>896262562</v>
+        <v>819807063</v>
       </c>
       <c r="I23" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J23" s="6" t="n">
-        <v>896262562</v>
+        <v>819807063</v>
       </c>
       <c r="K23" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>334523972</v>
+        <v>258068473</v>
       </c>
       <c r="M23" s="7" t="inlineStr">
         <is>
@@ -5860,28 +5882,28 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D25" s="6" t="n">
-        <v>1162285000</v>
+        <v>1042820000</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>966980500</v>
+        <v>847515500</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>962557890</v>
+        <v>847057950</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J25" s="6" t="n">
-        <v>962557890</v>
+        <v>847057950</v>
       </c>
       <c r="K25" s="7" t="inlineStr">
         <is>
@@ -5964,34 +5986,38 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D27" s="6" t="n">
-        <v>17749764478</v>
+        <v>17552967716</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F27" s="6" t="n">
-        <v>17749764478</v>
+        <v>17552967716</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>17474299910</v>
+        <v>17401334615</v>
       </c>
       <c r="I27" s="4" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J27" s="6" t="n">
-        <v>12559335992</v>
-      </c>
-      <c r="K27" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L27" s="6" t="n">
-        <v>72965295</v>
+        <v>12486370697</v>
+      </c>
+      <c r="K27" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L27" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M27" s="7" t="inlineStr">
         <is>
@@ -6014,28 +6040,28 @@
         </is>
       </c>
       <c r="C28" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D28" s="10" t="n">
-        <v>288750000</v>
+        <v>138750000</v>
       </c>
       <c r="E28" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F28" s="10" t="n">
-        <v>288750000</v>
+        <v>138750000</v>
       </c>
       <c r="G28" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H28" s="10" t="n">
-        <v>288306000</v>
+        <v>138306000</v>
       </c>
       <c r="I28" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J28" s="10" t="n">
-        <v>288306000</v>
+        <v>138306000</v>
       </c>
       <c r="K28" s="11" t="inlineStr">
         <is>
@@ -6071,13 +6097,13 @@
         <v>1</v>
       </c>
       <c r="D29" s="6" t="n">
-        <v>66310000</v>
+        <v>79572000</v>
       </c>
       <c r="E29" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F29" s="6" t="n">
-        <v>66310000</v>
+        <v>79572000</v>
       </c>
       <c r="G29" s="4" t="n">
         <v>1</v>
@@ -6284,28 +6310,28 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D33" s="6" t="n">
-        <v>886469138</v>
+        <v>1084801656</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F33" s="6" t="n">
-        <v>886469138</v>
+        <v>1084801656</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H33" s="6" t="n">
-        <v>823462550</v>
+        <v>1022541050</v>
       </c>
       <c r="I33" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J33" s="6" t="n">
-        <v>315286850</v>
+        <v>514365350</v>
       </c>
       <c r="K33" s="7" t="inlineStr">
         <is>
@@ -6341,13 +6367,13 @@
         <v>36</v>
       </c>
       <c r="D34" s="10" t="n">
-        <v>4775708657</v>
+        <v>4775292407</v>
       </c>
       <c r="E34" s="8" t="n">
         <v>36</v>
       </c>
       <c r="F34" s="10" t="n">
-        <v>4775708657</v>
+        <v>4775292407</v>
       </c>
       <c r="G34" s="8" t="n">
         <v>36</v>
@@ -6392,40 +6418,44 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="D35" s="6" t="n">
-        <v>2137090451</v>
+        <v>1487941951</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="F35" s="6" t="n">
-        <v>1951090451</v>
+        <v>1487941951</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="H35" s="6" t="n">
-        <v>1902420433</v>
+        <v>1444011523</v>
       </c>
       <c r="I35" s="4" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="J35" s="6" t="n">
-        <v>1692914483</v>
+        <v>1234505573</v>
       </c>
       <c r="K35" s="4" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="L35" s="6" t="n">
-        <v>713727983</v>
-      </c>
-      <c r="M35" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="N35" s="6" t="n">
-        <v>186000000</v>
+        <v>366519983</v>
+      </c>
+      <c r="M35" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N35" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="36" ht="45" customHeight="1">
@@ -6508,28 +6538,28 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D37" s="6" t="n">
-        <v>2769384586</v>
+        <v>2516286291</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F37" s="6" t="n">
-        <v>2674384586</v>
+        <v>2421286291</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="H37" s="6" t="n">
-        <v>2613571243</v>
+        <v>2388524693</v>
       </c>
       <c r="I37" s="4" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="J37" s="6" t="n">
-        <v>2438894693</v>
+        <v>2253924693</v>
       </c>
       <c r="K37" s="4" t="n">
         <v>1</v>
@@ -8046,28 +8076,28 @@
         </is>
       </c>
       <c r="C62" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D62" s="10" t="n">
-        <v>417917650</v>
+        <v>345935300</v>
       </c>
       <c r="E62" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F62" s="10" t="n">
-        <v>417917650</v>
+        <v>345935300</v>
       </c>
       <c r="G62" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H62" s="10" t="n">
-        <v>198768000</v>
+        <v>187868022</v>
       </c>
       <c r="I62" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J62" s="10" t="n">
-        <v>198768000</v>
+        <v>187868022</v>
       </c>
       <c r="K62" s="8" t="n">
         <v>2</v>
@@ -8220,28 +8250,28 @@
         </is>
       </c>
       <c r="C65" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D65" s="6" t="n">
-        <v>471330601</v>
+        <v>255172666</v>
       </c>
       <c r="E65" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F65" s="6" t="n">
-        <v>471330601</v>
+        <v>255172666</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H65" s="6" t="n">
-        <v>448555830</v>
+        <v>252188255</v>
       </c>
       <c r="I65" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J65" s="6" t="n">
-        <v>309615830</v>
+        <v>113248255</v>
       </c>
       <c r="K65" s="7" t="inlineStr">
         <is>
@@ -8762,34 +8792,38 @@
         </is>
       </c>
       <c r="C74" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D74" s="10" t="n">
-        <v>301830114</v>
+        <v>61977656</v>
       </c>
       <c r="E74" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F74" s="10" t="n">
-        <v>301830114</v>
+        <v>61977656</v>
       </c>
       <c r="G74" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H74" s="10" t="n">
-        <v>68020787</v>
+        <v>2619587</v>
       </c>
       <c r="I74" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J74" s="10" t="n">
-        <v>68020787</v>
-      </c>
-      <c r="K74" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="L74" s="10" t="n">
-        <v>65401200</v>
+        <v>2619587</v>
+      </c>
+      <c r="K74" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L74" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M74" s="11" t="inlineStr">
         <is>
@@ -10133,13 +10167,13 @@
         <v>1</v>
       </c>
       <c r="D96" s="10" t="n">
-        <v>146817603</v>
+        <v>115814581</v>
       </c>
       <c r="E96" s="8" t="n">
         <v>1</v>
       </c>
       <c r="F96" s="10" t="n">
-        <v>146817603</v>
+        <v>115814581</v>
       </c>
       <c r="G96" s="8" t="n">
         <v>1</v>
@@ -10412,28 +10446,28 @@
         </is>
       </c>
       <c r="C101" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="D101" s="6" t="n">
+        <v>789698247</v>
+      </c>
+      <c r="E101" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="D101" s="6" t="n">
-        <v>639698247</v>
-      </c>
-      <c r="E101" s="4" t="n">
-        <v>5</v>
-      </c>
       <c r="F101" s="6" t="n">
-        <v>564698247</v>
+        <v>714698247</v>
       </c>
       <c r="G101" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H101" s="6" t="n">
-        <v>552004825</v>
+        <v>701504825</v>
       </c>
       <c r="I101" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J101" s="6" t="n">
-        <v>552004825</v>
+        <v>701504825</v>
       </c>
       <c r="K101" s="7" t="inlineStr">
         <is>
@@ -10700,40 +10734,40 @@
         </is>
       </c>
       <c r="C106" s="12" t="n">
-        <v>890</v>
+        <v>872</v>
       </c>
       <c r="D106" s="13" t="n">
-        <v>105451667259</v>
+        <v>103645255356</v>
       </c>
       <c r="E106" s="12" t="n">
-        <v>531</v>
+        <v>514</v>
       </c>
       <c r="F106" s="13" t="n">
-        <v>66569520377</v>
+        <v>64949108474</v>
       </c>
       <c r="G106" s="12" t="n">
-        <v>531</v>
+        <v>514</v>
       </c>
       <c r="H106" s="13" t="n">
-        <v>64541638852</v>
+        <v>63469827355</v>
       </c>
       <c r="I106" s="12" t="n">
-        <v>373</v>
+        <v>357</v>
       </c>
       <c r="J106" s="13" t="n">
-        <v>46312544753</v>
+        <v>45280809806</v>
       </c>
       <c r="K106" s="12" t="n">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="L106" s="13" t="n">
-        <v>1796394590</v>
+        <v>1185019546</v>
       </c>
       <c r="M106" s="12" t="n">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="N106" s="13" t="n">
-        <v>38882146882</v>
+        <v>38696146882</v>
       </c>
     </row>
   </sheetData>
@@ -11955,34 +11989,34 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>33</v>
+        <v>8</v>
       </c>
       <c r="D23" s="6" t="n">
-        <v>49502018488</v>
+        <v>6785775489</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>33</v>
+        <v>8</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>49502018488</v>
+        <v>6785775489</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>33</v>
+        <v>8</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>5975304750</v>
+        <v>4647707037</v>
       </c>
       <c r="I23" s="4" t="n">
-        <v>33</v>
+        <v>8</v>
       </c>
       <c r="J23" s="6" t="n">
-        <v>5975304750</v>
+        <v>4647707037</v>
       </c>
       <c r="K23" s="4" t="n">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="L23" s="6" t="n">
-        <v>2945468782</v>
+        <v>1712457037</v>
       </c>
       <c r="M23" s="7" t="inlineStr">
         <is>
@@ -12183,28 +12217,28 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D27" s="6" t="n">
-        <v>35150142456</v>
+        <v>33347236056</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F27" s="6" t="n">
-        <v>35150142456</v>
+        <v>33347236056</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>34664094970</v>
+        <v>32867594970</v>
       </c>
       <c r="I27" s="4" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J27" s="6" t="n">
-        <v>33657050970</v>
+        <v>31860550970</v>
       </c>
       <c r="K27" s="7" t="inlineStr">
         <is>
@@ -12538,29 +12572,45 @@
           <t>DINAS PERHUBUNGAN - 2.15.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C33" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D33" s="6" t="n">
-        <v>201600000</v>
-      </c>
-      <c r="E33" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F33" s="6" t="n">
-        <v>201600000</v>
-      </c>
-      <c r="G33" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H33" s="6" t="n">
-        <v>199078500</v>
-      </c>
-      <c r="I33" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J33" s="6" t="n">
-        <v>199078500</v>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I33" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J33" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K33" s="7" t="inlineStr">
         <is>
@@ -12647,34 +12697,38 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D35" s="6" t="n">
-        <v>4037584000</v>
+        <v>2073094000</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F35" s="6" t="n">
-        <v>4037584000</v>
+        <v>2073094000</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H35" s="6" t="n">
-        <v>3591790630</v>
+        <v>2073094000</v>
       </c>
       <c r="I35" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J35" s="6" t="n">
-        <v>3591790630</v>
-      </c>
-      <c r="K35" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L35" s="6" t="n">
-        <v>436796630</v>
+        <v>2073094000</v>
+      </c>
+      <c r="K35" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L35" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M35" s="7" t="inlineStr">
         <is>
@@ -12767,28 +12821,28 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D37" s="6" t="n">
-        <v>3013841480</v>
+        <v>3162607980</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F37" s="6" t="n">
-        <v>3013841480</v>
+        <v>3162607980</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H37" s="6" t="n">
-        <v>2296738818</v>
+        <v>2481708818</v>
       </c>
       <c r="I37" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J37" s="6" t="n">
-        <v>2296738818</v>
+        <v>2481708818</v>
       </c>
       <c r="K37" s="4" t="n">
         <v>2</v>
@@ -12944,7 +12998,7 @@
         <v>2</v>
       </c>
       <c r="D40" s="10" t="n">
-        <v>520638000</v>
+        <v>515138000</v>
       </c>
       <c r="E40" s="8" t="n">
         <v>1</v>
@@ -12978,7 +13032,7 @@
         <v>1</v>
       </c>
       <c r="N40" s="10" t="n">
-        <v>277500000</v>
+        <v>272000000</v>
       </c>
     </row>
     <row r="41" ht="45" customHeight="1">
@@ -14306,13 +14360,13 @@
         <v>1</v>
       </c>
       <c r="D61" s="6" t="n">
-        <v>346000000</v>
+        <v>328338000</v>
       </c>
       <c r="E61" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F61" s="6" t="n">
-        <v>346000000</v>
+        <v>328338000</v>
       </c>
       <c r="G61" s="4" t="n">
         <v>1</v>
@@ -16735,28 +16789,28 @@
         </is>
       </c>
       <c r="C97" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D97" s="6" t="n">
-        <v>8054692000</v>
+        <v>1448692000</v>
       </c>
       <c r="E97" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F97" s="6" t="n">
-        <v>8054692000</v>
+        <v>1448692000</v>
       </c>
       <c r="G97" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H97" s="6" t="n">
-        <v>2808340212</v>
+        <v>607099212</v>
       </c>
       <c r="I97" s="4" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J97" s="6" t="n">
-        <v>2808340212</v>
+        <v>607099212</v>
       </c>
       <c r="K97" s="4" t="n">
         <v>2</v>
@@ -16987,28 +17041,28 @@
         </is>
       </c>
       <c r="C101" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D101" s="6" t="n">
-        <v>3294207800</v>
+        <v>2944207800</v>
       </c>
       <c r="E101" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F101" s="6" t="n">
-        <v>3294207800</v>
+        <v>2944207800</v>
       </c>
       <c r="G101" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H101" s="6" t="n">
-        <v>3091941500</v>
+        <v>2942441500</v>
       </c>
       <c r="I101" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J101" s="6" t="n">
-        <v>2207941500</v>
+        <v>2058441500</v>
       </c>
       <c r="K101" s="7" t="inlineStr">
         <is>
@@ -17279,40 +17333,40 @@
         </is>
       </c>
       <c r="C106" s="12" t="n">
-        <v>240</v>
+        <v>208</v>
       </c>
       <c r="D106" s="13" t="n">
-        <v>181564348470</v>
+        <v>128048713571</v>
       </c>
       <c r="E106" s="12" t="n">
-        <v>162</v>
+        <v>130</v>
       </c>
       <c r="F106" s="13" t="n">
-        <v>147176925531</v>
+        <v>93666790632</v>
       </c>
       <c r="G106" s="12" t="n">
-        <v>162</v>
+        <v>130</v>
       </c>
       <c r="H106" s="13" t="n">
-        <v>71920708305</v>
+        <v>64913064462</v>
       </c>
       <c r="I106" s="12" t="n">
-        <v>149</v>
+        <v>117</v>
       </c>
       <c r="J106" s="13" t="n">
-        <v>67648469205</v>
+        <v>60640825362</v>
       </c>
       <c r="K106" s="12" t="n">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="L106" s="13" t="n">
-        <v>4430709261</v>
+        <v>2760900886</v>
       </c>
       <c r="M106" s="12" t="n">
         <v>78</v>
       </c>
       <c r="N106" s="13" t="n">
-        <v>34387422939</v>
+        <v>34381922939</v>
       </c>
     </row>
   </sheetData>
@@ -18663,29 +18717,45 @@
           <t>DINAS KOMUNIKASI, INFORMATIKA, STATISTIK DAN PERSANDIAN - 2.16.2.20.2.21.01.0000</t>
         </is>
       </c>
-      <c r="C24" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D24" s="10" t="n">
-        <v>2700000000</v>
-      </c>
-      <c r="E24" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F24" s="10" t="n">
-        <v>2700000000</v>
-      </c>
-      <c r="G24" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="H24" s="10" t="n">
-        <v>2699298000</v>
-      </c>
-      <c r="I24" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="J24" s="10" t="n">
-        <v>2699298000</v>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K24" s="11" t="inlineStr">
         <is>
@@ -19249,13 +19319,13 @@
         <v>1</v>
       </c>
       <c r="D33" s="6" t="n">
-        <v>5040000000</v>
+        <v>4988300000</v>
       </c>
       <c r="E33" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F33" s="6" t="n">
-        <v>5040000000</v>
+        <v>4988300000</v>
       </c>
       <c r="G33" s="4" t="n">
         <v>1</v>
@@ -19369,29 +19439,45 @@
           <t>DINAS PERINDUSTRIAN, PERDAGANGAN, KOPERASI, USAHA KECIL DAN MENENGAH - 2.17.3.30.3.31.01.0000</t>
         </is>
       </c>
-      <c r="C35" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D35" s="6" t="n">
-        <v>2688000000</v>
-      </c>
-      <c r="E35" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F35" s="6" t="n">
-        <v>2688000000</v>
-      </c>
-      <c r="G35" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H35" s="6" t="n">
-        <v>2646500000</v>
-      </c>
-      <c r="I35" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J35" s="6" t="n">
-        <v>2646500000</v>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I35" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J35" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K35" s="7" t="inlineStr">
         <is>
@@ -24258,28 +24344,28 @@
         </is>
       </c>
       <c r="C106" s="12" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D106" s="13" t="n">
-        <v>251072475553</v>
+        <v>245632775553</v>
       </c>
       <c r="E106" s="12" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F106" s="13" t="n">
-        <v>147115370800</v>
+        <v>141675670800</v>
       </c>
       <c r="G106" s="12" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="H106" s="13" t="n">
-        <v>71235380009</v>
+        <v>65889582009</v>
       </c>
       <c r="I106" s="12" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="J106" s="13" t="n">
-        <v>71235380009</v>
+        <v>65889582009</v>
       </c>
       <c r="K106" s="2" t="inlineStr">
         <is>

</xml_diff>